<commit_message>
chore: fill in the three remaining last-rotated dates
SENTRY_AUTH_TOKEN: 3 Sep 2026 · TURNSTILE_SECRET_KEY: 17 Aug 2026 ·
INFRA_VERCEL_TOKEN: 3 Sep 2026 — supplied by AJ.

All 17 tracked secrets now have a real last-rotated date and current
status. Nothing overdue or due soon; every row reads ✓ OK.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -15,9 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -1037,14 +1035,16 @@
       <c r="D18" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="9" t="str">
+      <c r="E18" s="8" t="n">
+        <v>46268</v>
+      </c>
+      <c r="F18" s="9">
         <f>IFERROR(IF(E18="","",EDATE(E18,D18)),"")</f>
-        <v/>
+        <v>46633</v>
       </c>
       <c r="G18" s="6" t="str">
         <f>IFERROR(IF(F18="","Not set",IF(F18&lt;TODAY(),"⚠ OVERDUE",IF(F18&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>Not set</v>
+        <v>✓ OK</v>
       </c>
     </row>
     <row r="19">
@@ -1066,14 +1066,16 @@
       <c r="D19" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="9" t="str">
+      <c r="E19" s="8" t="n">
+        <v>46251</v>
+      </c>
+      <c r="F19" s="9">
         <f>IFERROR(IF(E19="","",EDATE(E19,D19)),"")</f>
-        <v/>
+        <v>46616</v>
       </c>
       <c r="G19" s="6" t="str">
         <f>IFERROR(IF(F19="","Not set",IF(F19&lt;TODAY(),"⚠ OVERDUE",IF(F19&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>Not set</v>
+        <v>✓ OK</v>
       </c>
     </row>
     <row r="20">
@@ -1095,14 +1097,16 @@
       <c r="D20" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="9" t="str">
+      <c r="E20" s="8" t="n">
+        <v>46268</v>
+      </c>
+      <c r="F20" s="9">
         <f>IFERROR(IF(E20="","",EDATE(E20,D20)),"")</f>
-        <v/>
+        <v>46633</v>
       </c>
       <c r="G20" s="6" t="str">
         <f>IFERROR(IF(F20="","Not set",IF(F20&lt;TODAY(),"⚠ OVERDUE",IF(F20&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>Not set</v>
+        <v>✓ OK</v>
       </c>
     </row>
     <row r="21">
@@ -1112,8 +1116,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Generate the e2e cron secret per run; log CRON_SECRET rotation
- playwright.config.ts now generates a random CRON_SECRET for every test run
  (32 random bytes, hex), passes it to the dev server and shares it with the
  specs through E2E_CRON_SECRET, read back in e2e/support/cron.ts. The
  repository is public, so it no longer contains a fixed value that looks
  like a credential. e2e/support/cron.ts fails with a clear message if the
  variable is missing.
- docs/alwaysready-api-key-rotation-log.xlsx: CRON_SECRET last rotated
  2026-09-20 (production value replaced in Vercel; next due 2027-09-20).
  Only that date and its cached next-due result changed in the workbook.

All 13 specs that use the secret pass on three consecutive runs from a
fresh seed; the full suite passes 68/68 (subscribe.spec excluded, it needs
a live `stripe listen`).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -850,11 +850,11 @@
         <v>12</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46219</v>
+        <v>46285</v>
       </c>
       <c r="F12" s="9">
         <f>IFERROR(IF(E12="","",EDATE(E12,D12)),"")</f>
-        <v>46584</v>
+        <v>46650</v>
       </c>
       <c r="G12" s="6" t="str">
         <f>IFERROR(IF(F12="","Not set",IF(F12&lt;TODAY(),"⚠ OVERDUE",IF(F12&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>

</xml_diff>

<commit_message>
Tidy env keys after removing AI drafts and demo bookings
ANTHROPIC_API_KEY and ZEEG_WEBHOOK_TOKEN are no longer read by any code,
so drop them from .env.example, the CI placeholder env, and the rotation
log. Add the four R2_* names (read by the storage-backup cron) to
.env.example, and record the four R2 keys in the rotation log.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -606,11 +606,11 @@
       </c>
       <c r="F4" s="9">
         <f>IFERROR(IF(E4="","",EDATE(E4,D4)),"")</f>
-        <v>46583</v>
-      </c>
-      <c r="G4" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G4" s="6">
         <f>IFERROR(IF(F4="","Not set",IF(F4&lt;TODAY(),"⚠ OVERDUE",IF(F4&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
@@ -637,11 +637,11 @@
       </c>
       <c r="F5" s="13">
         <f>IFERROR(IF(E5="","",EDATE(E5,D5)),"")</f>
-        <v>46402</v>
-      </c>
-      <c r="G5" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="11">
         <f>IFERROR(IF(F5="","Not set",IF(F5&lt;TODAY(),"⚠ OVERDUE",IF(F5&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -668,11 +668,11 @@
       </c>
       <c r="F6" s="9">
         <f>IFERROR(IF(E6="","",EDATE(E6,D6)),"")</f>
-        <v>46585</v>
-      </c>
-      <c r="G6" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G6" s="6">
         <f>IFERROR(IF(F6="","Not set",IF(F6&lt;TODAY(),"⚠ OVERDUE",IF(F6&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
@@ -699,11 +699,11 @@
       </c>
       <c r="F7" s="13">
         <f>IFERROR(IF(E7="","",EDATE(E7,D7)),"")</f>
-        <v>46595</v>
-      </c>
-      <c r="G7" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="11">
         <f>IFERROR(IF(F7="","Not set",IF(F7&lt;TODAY(),"⚠ OVERDUE",IF(F7&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
@@ -730,244 +730,244 @@
       </c>
       <c r="F8" s="9">
         <f>IFERROR(IF(E8="","",EDATE(E8,D8)),"")</f>
-        <v>46595</v>
-      </c>
-      <c r="G8" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="6">
         <f>IFERROR(IF(F8="","Not set",IF(F8&lt;TODAY(),"⚠ OVERDUE",IF(F8&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>console.anthropic.com → API Keys → Create new → delete old</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>CLOUDMERSIVE_API_KEY</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Cloudmersive</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46240</v>
-      </c>
-      <c r="F9" s="13">
+        <v>46220</v>
+      </c>
+      <c r="F9" s="9">
         <f>IFERROR(IF(E9="","",EDATE(E9,D9)),"")</f>
-        <v>46605</v>
-      </c>
-      <c r="G9" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G9" s="6">
         <f>IFERROR(IF(F9="","Not set",IF(F9&lt;TODAY(),"⚠ OVERDUE",IF(F9&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>CLOUDMERSIVE_API_KEY</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Cloudmersive</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>INBOUND_EMAIL_SECRET</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>openssl rand -hex 32 → update Vercel + Cloudflare Worker</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46220</v>
-      </c>
-      <c r="F10" s="9">
+        <v>46231</v>
+      </c>
+      <c r="F10" s="13">
         <f>IFERROR(IF(E10="","",EDATE(E10,D10)),"")</f>
-        <v>46585</v>
-      </c>
-      <c r="G10" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G10" s="11">
         <f>IFERROR(IF(F10="","Not set",IF(F10&lt;TODAY(),"⚠ OVERDUE",IF(F10&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>INBOUND_EMAIL_SECRET</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Self-generated</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>openssl rand -hex 32 → update Vercel + Cloudflare Worker</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="n">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>openssl rand -hex 32 → update Vercel env var</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46231</v>
-      </c>
-      <c r="F11" s="13">
+        <v>46285</v>
+      </c>
+      <c r="F11" s="9">
         <f>IFERROR(IF(E11="","",EDATE(E11,D11)),"")</f>
-        <v>46596</v>
-      </c>
-      <c r="G11" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G11" s="6">
         <f>IFERROR(IF(F11="","Not set",IF(F11&lt;TODAY(),"⚠ OVERDUE",IF(F11&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>CRON_SECRET</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>UNSUBSCRIBE_SECRET</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Self-generated</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>openssl rand -hex 32 → update Vercel env var</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F12" s="9">
+        <v>46221</v>
+      </c>
+      <c r="F12" s="13">
         <f>IFERROR(IF(E12="","",EDATE(E12,D12)),"")</f>
-        <v>46650</v>
-      </c>
-      <c r="G12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G12" s="11">
         <f>IFERROR(IF(F12="","Not set",IF(F12&lt;TODAY(),"⚠ OVERDUE",IF(F12&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>UNSUBSCRIBE_SECRET</t>
+          <t>UPSTASH_REDIS_REST_TOKEN</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Self-generated</t>
+          <t>Upstash</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>openssl rand -hex 32 → update Vercel env var</t>
+          <t>console.upstash.com → Redis → REST API → Reset token</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>46221</v>
+        <v>46257</v>
       </c>
       <c r="F13" s="13">
         <f>IFERROR(IF(E13="","",EDATE(E13,D13)),"")</f>
-        <v>46586</v>
-      </c>
-      <c r="G13" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G13" s="11">
         <f>IFERROR(IF(F13="","Not set",IF(F13&lt;TODAY(),"⚠ OVERDUE",IF(F13&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>ZEEG_WEBHOOK_TOKEN</t>
+          <t>UPSTASH_MANAGEMENT_API_KEY</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Zeeg</t>
+          <t>Upstash</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Zeeg dashboard → Webhooks → Regenerate token</t>
+          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>46236</v>
+        <v>46268</v>
       </c>
       <c r="F14" s="9">
         <f>IFERROR(IF(E14="","",EDATE(E14,D14)),"")</f>
-        <v>46601</v>
-      </c>
-      <c r="G14" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G14" s="6">
         <f>IFERROR(IF(F14="","Not set",IF(F14&lt;TODAY(),"⚠ OVERDUE",IF(F14&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>UPSTASH_REDIS_REST_TOKEN</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Upstash</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>console.upstash.com → Redis → REST API → Reset token</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_API_TOKEN</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46257</v>
-      </c>
-      <c r="F15" s="13">
+        <v>46268</v>
+      </c>
+      <c r="F15" s="9">
         <f>IFERROR(IF(E15="","",EDATE(E15,D15)),"")</f>
-        <v>46622</v>
-      </c>
-      <c r="G15" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G15" s="6">
         <f>IFERROR(IF(F15="","Not set",IF(F15&lt;TODAY(),"⚠ OVERDUE",IF(F15&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>UPSTASH_MANAGEMENT_API_KEY</t>
+          <t>SENTRY_AUTH_TOKEN</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Upstash</t>
+          <t>Sentry</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
+          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -978,58 +978,58 @@
       </c>
       <c r="F16" s="9">
         <f>IFERROR(IF(E16="","",EDATE(E16,D16)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G16" s="6">
         <f>IFERROR(IF(F16="","Not set",IF(F16&lt;TODAY(),"⚠ OVERDUE",IF(F16&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="21.75" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>CLOUDFLARE_API_TOKEN</t>
+          <t>TURNSTILE_SECRET_KEY</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Cloudflare Turnstile</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46268</v>
+        <v>46251</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(IF(E17="","",EDATE(E17,D17)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G17" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G17" s="6">
         <f>IFERROR(IF(F17="","Not set",IF(F17&lt;TODAY(),"⚠ OVERDUE",IF(F17&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>SENTRY_AUTH_TOKEN</t>
+          <t>INFRA_VERCEL_TOKEN</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Sentry</t>
+          <t>Vercel</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
+          <t>vercel.com/account/tokens → delete old → create new</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -1040,119 +1040,175 @@
       </c>
       <c r="F18" s="9">
         <f>IFERROR(IF(E18="","",EDATE(E18,D18)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G18" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G18" s="6">
         <f>IFERROR(IF(F18="","Not set",IF(F18&lt;TODAY(),"⚠ OVERDUE",IF(F18&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>TURNSTILE_SECRET_KEY</t>
+          <t>R2_ACCOUNT_ID</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Cloudflare Turnstile</t>
+          <t>Cloudflare R2</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>46251</v>
-      </c>
+          <t>Fixed account identifier, not a rotating secret (Cloudflare account ID)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="8" t="n"/>
       <c r="F19" s="9">
         <f>IFERROR(IF(E19="","",EDATE(E19,D19)),"")</f>
-        <v>46616</v>
-      </c>
-      <c r="G19" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G19" s="6">
         <f>IFERROR(IF(F19="","Not set",IF(F19&lt;TODAY(),"⚠ OVERDUE",IF(F19&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>INFRA_VERCEL_TOKEN</t>
+          <t>R2_ACCESS_KEY_ID</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Cloudflare R2</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>vercel.com/account/tokens → delete old → create new</t>
+          <t>dash.cloudflare.com → R2 Object Storage → Manage API Tokens → delete old → Create Account API token (Object Read &amp; Write, scoped to alwaysready-storage-backup)</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46268</v>
+        <v>46287</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(IF(E20="","",EDATE(E20,D20)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G20" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G20" s="6">
         <f>IFERROR(IF(F20="","Not set",IF(F20&lt;TODAY(),"⚠ OVERDUE",IF(F20&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>R2_SECRET_ACCESS_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Same API token as R2_ACCESS_KEY_ID, regenerate and update both together</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="F21" s="9">
+        <f>IFERROR(IF(E21="","",EDATE(E21,D21)),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="6">
+        <f>IFERROR(IF(F21="","Not set",IF(F21&lt;TODAY(),"⚠ OVERDUE",IF(F21&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>R2_BUCKET_NAME</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Fixed bucket name, not a rotating secret</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="9">
+        <f>IFERROR(IF(E22="","",EDATE(E22,D22)),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="6">
+        <f>IFERROR(IF(F22="","Not set",IF(F22&lt;TODAY(),"⚠ OVERDUE",IF(F22&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>🟡 Yellow cells = enter date here    |    ⚠ OVERDUE = rotation is past due    |    Due soon = within 30 days    |    ✓ OK = rotation is current</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Supabase Anon Key — safe to rotate; triggers a brief auth token refresh for logged-in users.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Supabase Service Role Key — rotate with care; used server-side only. Update Vercel env var and redeploy immediately after.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Self-generated secrets (INBOUND_EMAIL_SECRET, CRON_SECRET, UNSUBSCRIBE_SECRET) — generate with: openssl rand -hex 32</t>
+          <t>Supabase Anon Key — safe to rotate; triggers a brief auth token refresh for logged-in users.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Stripe Secret Key — Stripe supports zero-downtime rolling: generate new key, update Vercel, verify, then revoke old.</t>
+          <t>Supabase Service Role Key — rotate with care; used server-side only. Update Vercel env var and redeploy immediately after.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Self-generated secrets (INBOUND_EMAIL_SECRET, CRON_SECRET, UNSUBSCRIBE_SECRET) — generate with: openssl rand -hex 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Stripe Secret Key — Stripe supports zero-downtime rolling: generate new key, update Vercel, verify, then revoke old.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Upstash Redis Token — resetting the token invalidates all existing connections immediately; update Vercel and redeploy straight away.</t>
         </is>

</xml_diff>

<commit_message>
Tidy env keys after removing AI drafts and demo bookings (#73)
ANTHROPIC_API_KEY and ZEEG_WEBHOOK_TOKEN are no longer read by any code,
so drop them from .env.example, the CI placeholder env, and the rotation
log. Add the four R2_* names (read by the storage-backup cron) to
.env.example, and record the four R2 keys in the rotation log.

Co-authored-by: AJ Parker <ethnainiceland@gmail.com>
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -606,11 +606,11 @@
       </c>
       <c r="F4" s="9">
         <f>IFERROR(IF(E4="","",EDATE(E4,D4)),"")</f>
-        <v>46583</v>
-      </c>
-      <c r="G4" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G4" s="6">
         <f>IFERROR(IF(F4="","Not set",IF(F4&lt;TODAY(),"⚠ OVERDUE",IF(F4&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
@@ -637,11 +637,11 @@
       </c>
       <c r="F5" s="13">
         <f>IFERROR(IF(E5="","",EDATE(E5,D5)),"")</f>
-        <v>46402</v>
-      </c>
-      <c r="G5" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="11">
         <f>IFERROR(IF(F5="","Not set",IF(F5&lt;TODAY(),"⚠ OVERDUE",IF(F5&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
@@ -668,11 +668,11 @@
       </c>
       <c r="F6" s="9">
         <f>IFERROR(IF(E6="","",EDATE(E6,D6)),"")</f>
-        <v>46585</v>
-      </c>
-      <c r="G6" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G6" s="6">
         <f>IFERROR(IF(F6="","Not set",IF(F6&lt;TODAY(),"⚠ OVERDUE",IF(F6&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
@@ -699,11 +699,11 @@
       </c>
       <c r="F7" s="13">
         <f>IFERROR(IF(E7="","",EDATE(E7,D7)),"")</f>
-        <v>46595</v>
-      </c>
-      <c r="G7" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="11">
         <f>IFERROR(IF(F7="","Not set",IF(F7&lt;TODAY(),"⚠ OVERDUE",IF(F7&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
@@ -730,244 +730,244 @@
       </c>
       <c r="F8" s="9">
         <f>IFERROR(IF(E8="","",EDATE(E8,D8)),"")</f>
-        <v>46595</v>
-      </c>
-      <c r="G8" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="6">
         <f>IFERROR(IF(F8="","Not set",IF(F8&lt;TODAY(),"⚠ OVERDUE",IF(F8&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>ANTHROPIC_API_KEY</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Anthropic</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>console.anthropic.com → API Keys → Create new → delete old</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="n">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>CLOUDMERSIVE_API_KEY</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Cloudmersive</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46240</v>
-      </c>
-      <c r="F9" s="13">
+        <v>46220</v>
+      </c>
+      <c r="F9" s="9">
         <f>IFERROR(IF(E9="","",EDATE(E9,D9)),"")</f>
-        <v>46605</v>
-      </c>
-      <c r="G9" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G9" s="6">
         <f>IFERROR(IF(F9="","Not set",IF(F9&lt;TODAY(),"⚠ OVERDUE",IF(F9&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>CLOUDMERSIVE_API_KEY</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Cloudmersive</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>INBOUND_EMAIL_SECRET</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>openssl rand -hex 32 → update Vercel + Cloudflare Worker</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46220</v>
-      </c>
-      <c r="F10" s="9">
+        <v>46231</v>
+      </c>
+      <c r="F10" s="13">
         <f>IFERROR(IF(E10="","",EDATE(E10,D10)),"")</f>
-        <v>46585</v>
-      </c>
-      <c r="G10" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G10" s="11">
         <f>IFERROR(IF(F10="","Not set",IF(F10&lt;TODAY(),"⚠ OVERDUE",IF(F10&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>INBOUND_EMAIL_SECRET</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Self-generated</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>openssl rand -hex 32 → update Vercel + Cloudflare Worker</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="n">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>openssl rand -hex 32 → update Vercel env var</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46231</v>
-      </c>
-      <c r="F11" s="13">
+        <v>46285</v>
+      </c>
+      <c r="F11" s="9">
         <f>IFERROR(IF(E11="","",EDATE(E11,D11)),"")</f>
-        <v>46596</v>
-      </c>
-      <c r="G11" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G11" s="6">
         <f>IFERROR(IF(F11="","Not set",IF(F11&lt;TODAY(),"⚠ OVERDUE",IF(F11&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>CRON_SECRET</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>UNSUBSCRIBE_SECRET</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Self-generated</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>openssl rand -hex 32 → update Vercel env var</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F12" s="9">
+        <v>46221</v>
+      </c>
+      <c r="F12" s="13">
         <f>IFERROR(IF(E12="","",EDATE(E12,D12)),"")</f>
-        <v>46650</v>
-      </c>
-      <c r="G12" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G12" s="11">
         <f>IFERROR(IF(F12="","Not set",IF(F12&lt;TODAY(),"⚠ OVERDUE",IF(F12&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>UNSUBSCRIBE_SECRET</t>
+          <t>UPSTASH_REDIS_REST_TOKEN</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Self-generated</t>
+          <t>Upstash</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>openssl rand -hex 32 → update Vercel env var</t>
+          <t>console.upstash.com → Redis → REST API → Reset token</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
         <v>12</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>46221</v>
+        <v>46257</v>
       </c>
       <c r="F13" s="13">
         <f>IFERROR(IF(E13="","",EDATE(E13,D13)),"")</f>
-        <v>46586</v>
-      </c>
-      <c r="G13" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G13" s="11">
         <f>IFERROR(IF(F13="","Not set",IF(F13&lt;TODAY(),"⚠ OVERDUE",IF(F13&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>ZEEG_WEBHOOK_TOKEN</t>
+          <t>UPSTASH_MANAGEMENT_API_KEY</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Zeeg</t>
+          <t>Upstash</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Zeeg dashboard → Webhooks → Regenerate token</t>
+          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>46236</v>
+        <v>46268</v>
       </c>
       <c r="F14" s="9">
         <f>IFERROR(IF(E14="","",EDATE(E14,D14)),"")</f>
-        <v>46601</v>
-      </c>
-      <c r="G14" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G14" s="6">
         <f>IFERROR(IF(F14="","Not set",IF(F14&lt;TODAY(),"⚠ OVERDUE",IF(F14&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>UPSTASH_REDIS_REST_TOKEN</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Upstash</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>console.upstash.com → Redis → REST API → Reset token</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_API_TOKEN</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46257</v>
-      </c>
-      <c r="F15" s="13">
+        <v>46268</v>
+      </c>
+      <c r="F15" s="9">
         <f>IFERROR(IF(E15="","",EDATE(E15,D15)),"")</f>
-        <v>46622</v>
-      </c>
-      <c r="G15" s="11" t="str">
+        <v/>
+      </c>
+      <c r="G15" s="6">
         <f>IFERROR(IF(F15="","Not set",IF(F15&lt;TODAY(),"⚠ OVERDUE",IF(F15&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>UPSTASH_MANAGEMENT_API_KEY</t>
+          <t>SENTRY_AUTH_TOKEN</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Upstash</t>
+          <t>Sentry</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
+          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -978,58 +978,58 @@
       </c>
       <c r="F16" s="9">
         <f>IFERROR(IF(E16="","",EDATE(E16,D16)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G16" s="6">
         <f>IFERROR(IF(F16="","Not set",IF(F16&lt;TODAY(),"⚠ OVERDUE",IF(F16&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="17" ht="21.75" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>CLOUDFLARE_API_TOKEN</t>
+          <t>TURNSTILE_SECRET_KEY</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Cloudflare Turnstile</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46268</v>
+        <v>46251</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(IF(E17="","",EDATE(E17,D17)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G17" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G17" s="6">
         <f>IFERROR(IF(F17="","Not set",IF(F17&lt;TODAY(),"⚠ OVERDUE",IF(F17&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="18" ht="19.5" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>SENTRY_AUTH_TOKEN</t>
+          <t>INFRA_VERCEL_TOKEN</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Sentry</t>
+          <t>Vercel</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
+          <t>vercel.com/account/tokens → delete old → create new</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -1040,119 +1040,175 @@
       </c>
       <c r="F18" s="9">
         <f>IFERROR(IF(E18="","",EDATE(E18,D18)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G18" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G18" s="6">
         <f>IFERROR(IF(F18="","Not set",IF(F18&lt;TODAY(),"⚠ OVERDUE",IF(F18&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>TURNSTILE_SECRET_KEY</t>
+          <t>R2_ACCOUNT_ID</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Cloudflare Turnstile</t>
+          <t>Cloudflare R2</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>46251</v>
-      </c>
+          <t>Fixed account identifier, not a rotating secret (Cloudflare account ID)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="8" t="n"/>
       <c r="F19" s="9">
         <f>IFERROR(IF(E19="","",EDATE(E19,D19)),"")</f>
-        <v>46616</v>
-      </c>
-      <c r="G19" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G19" s="6">
         <f>IFERROR(IF(F19="","Not set",IF(F19&lt;TODAY(),"⚠ OVERDUE",IF(F19&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>INFRA_VERCEL_TOKEN</t>
+          <t>R2_ACCESS_KEY_ID</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Cloudflare R2</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>vercel.com/account/tokens → delete old → create new</t>
+          <t>dash.cloudflare.com → R2 Object Storage → Manage API Tokens → delete old → Create Account API token (Object Read &amp; Write, scoped to alwaysready-storage-backup)</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
         <v>12</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46268</v>
+        <v>46287</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(IF(E20="","",EDATE(E20,D20)),"")</f>
-        <v>46633</v>
-      </c>
-      <c r="G20" s="6" t="str">
+        <v/>
+      </c>
+      <c r="G20" s="6">
         <f>IFERROR(IF(F20="","Not set",IF(F20&lt;TODAY(),"⚠ OVERDUE",IF(F20&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
-        <v>✓ OK</v>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>R2_SECRET_ACCESS_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Same API token as R2_ACCESS_KEY_ID, regenerate and update both together</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="F21" s="9">
+        <f>IFERROR(IF(E21="","",EDATE(E21,D21)),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="6">
+        <f>IFERROR(IF(F21="","Not set",IF(F21&lt;TODAY(),"⚠ OVERDUE",IF(F21&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>R2_BUCKET_NAME</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Fixed bucket name, not a rotating secret</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="9">
+        <f>IFERROR(IF(E22="","",EDATE(E22,D22)),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="6">
+        <f>IFERROR(IF(F22="","Not set",IF(F22&lt;TODAY(),"⚠ OVERDUE",IF(F22&lt;=TODAY()+30,"Due soon","✓ OK"))),"Not set")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>🟡 Yellow cells = enter date here    |    ⚠ OVERDUE = rotation is past due    |    Due soon = within 30 days    |    ✓ OK = rotation is current</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Supabase Anon Key — safe to rotate; triggers a brief auth token refresh for logged-in users.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Supabase Service Role Key — rotate with care; used server-side only. Update Vercel env var and redeploy immediately after.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Self-generated secrets (INBOUND_EMAIL_SECRET, CRON_SECRET, UNSUBSCRIBE_SECRET) — generate with: openssl rand -hex 32</t>
+          <t>Supabase Anon Key — safe to rotate; triggers a brief auth token refresh for logged-in users.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>Stripe Secret Key — Stripe supports zero-downtime rolling: generate new key, update Vercel, verify, then revoke old.</t>
+          <t>Supabase Service Role Key — rotate with care; used server-side only. Update Vercel env var and redeploy immediately after.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Self-generated secrets (INBOUND_EMAIL_SECRET, CRON_SECRET, UNSUBSCRIBE_SECRET) — generate with: openssl rand -hex 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Stripe Secret Key — Stripe supports zero-downtime rolling: generate new key, update Vercel, verify, then revoke old.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Upstash Redis Token — resetting the token invalidates all existing connections immediately; update Vercel and redeploy straight away.</t>
         </is>

</xml_diff>

<commit_message>
Add a Recovery Guide tab: where every environment variable lives
Vercel hides production secrets once saved, so recovery means regenerating,
not restoring. The new tab lists all 36 variables the platform reads, whether
each is a secret or a setting, where it is stored, how to get it back, and
what to know when replacing it, plus a rebuild checklist. It holds no values.
backup-and-recovery.md points to it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Key Rotation Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recovery Guide" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -16,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -80,8 +81,25 @@
       <color rgb="001A1A1A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF014D4E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF014D4E"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +148,23 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF014D4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -198,11 +231,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8D4D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8D4D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB8D4D4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB8D4D4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -257,6 +304,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1214,6 +1281,14 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -1222,4 +1297,1291 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>AlwaysReady Platform: Where every setting lives and how to get it back</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>This sheet holds no secret values, only where each one is stored and how to replace it. Vercel hides production secrets once saved, so the plan if something is lost is to regenerate, never to restore from a copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Secret or setting</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Stored in</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>How to get it back</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>What to know when you replace it</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Supabase dashboard, production project (alwaysready-production). Do not use the preview project's address.</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy after changing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_ANON_KEY</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Dashboard → Project Settings → API → Roll</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Logged-in users get a brief auth token refresh. Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>SUPABASE_SERVICE_ROLE_KEY</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Dashboard → Project Settings → API → Roll</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Server-side only. Update Vercel and redeploy straight away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_SECRET_KEY</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>dashboard.stripe.com → Developers → API keys → Roll key</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Stripe supports rolling: create the new key, update Vercel, verify, then revoke the old one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>STRIPE_WEBHOOK_SECRET</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>dashboard.stripe.com → Developers → Webhooks → Roll secret</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Payment and subscription updates fail to verify until Vercel has the new value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the standard plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only. If a price is recreated its ID changes and Vercel must be updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>STRIPE_CHARITY_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the charity plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_BETA_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the beta plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>resend.com → API Keys → Create new → delete old</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>No email sends until Vercel has the new key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>RESEND_FROM_ADDRESS</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Your own sender address. See .env.example for the expected format.</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>RESEND_REPLY_TO</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Your own reply-to address. See .env.example.</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>No side effects. Vercel sends it to scheduled jobs automatically after a redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>INBOUND_EMAIL_SECRET</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables) AND the Cloudflare Worker that forwards inbound email</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Set the SAME new value in both places, or customer email replies stop reaching the platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>UNSUBSCRIBE_SECRET</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>Every unsubscribe link already sent in past emails stops working, because links are signed with this secret. Only replace if it is lost or leaked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>CLOUDMERSIVE_API_KEY</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>Cloudmersive</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Update Vercel and redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_TURNSTILE_SITE_KEY</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile: the widget used by the platform. It is a pair with TURNSTILE_SECRET_KEY.</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy. Must belong to the same widget as the secret key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>TURNSTILE_SECRET_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>Bot check on sign-up forms fails until Vercel matches the widget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SENTRY_DSN</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Sentry: the platform project's client key (DSN).</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>Public by design. Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>SENTRY_ORG_SLUG</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Sentry organisation name (alwaysready-platform, per .env.example).</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>SENTRY_AUTH_TOKEN</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_REST_URL</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Upstash: the Redis database's REST address.</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_REST_TOKEN</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>console.upstash.com → Redis → REST API → Reset token</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>Resetting invalidates existing connections immediately. Update Vercel and redeploy straight away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_MANAGEMENT_API_KEY</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>UPSTASH_MANAGEMENT_EMAIL</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Your Upstash account email.</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_DATABASE_ID</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Upstash: the Redis database's ID.</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>INFRA_VERCEL_TOKEN</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>vercel.com/account/tokens → delete old → create new</t>
+        </is>
+      </c>
+      <c r="F30" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>INFRA_VERCEL_TEAM_ID</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel: your team's ID.</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_API_TOKEN</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+        </is>
+      </c>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_ACCOUNT_ID</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare: your account ID.</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>A wrong value here previously blanked the Infrastructure card. Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_WORKER_NAME</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare: the name of the email Worker.</t>
+        </is>
+      </c>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>A wrong value here previously blanked the Infrastructure card. Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>R2_ACCOUNT_ID</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare: your account ID (same as CLOUDFLARE_ACCOUNT_ID).</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>R2_ACCESS_KEY_ID</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → R2 Object Storage → Manage API Tokens → delete old → Create Account API token (Object Read &amp; Write, scoped to alwaysready-storage-backup)</t>
+        </is>
+      </c>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <t>Nightly Storage backup stops until Vercel has the new pair. /api/health reports it after about 27 hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>R2_SECRET_ACCESS_KEY</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>Same API token as R2_ACCESS_KEY_ID, regenerate and update both together</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>Comes as a pair with R2_ACCESS_KEY_ID: replace both together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>R2_BUCKET_NAME</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>alwaysready-storage-backup (the bucket's name).</t>
+        </is>
+      </c>
+      <c r="F38" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SITE_URL</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Own domain</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>The platform's public address (see .env.example).</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>SUPERADMIN_EMAIL</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>Own domain</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>Your superadmin email (see .env.example).</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>If the Vercel project or its variables are ever lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>0. First, make sure you can log in to every service listed above (keep each two-step recovery code safe). Without access, nothing can be regenerated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>1. Restore or recreate the Vercel project and connect the GitHub repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>2. Add every row marked Setting, looking each up as described in "How to get it back".</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>3. For every row marked Secret: regenerate it at its own service, or generate a new value for the self-generated ones, then add it to Vercel. INBOUND_EMAIL_SECRET also goes into the Cloudflare Worker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>4. Redeploy so the new values take effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>5. Check: /api/health returns 200; you can sign in; a test payment event reaches the platform; an email sends; the nightly Storage backup runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>6. Record the new dates in the "Last rotated" column on the Key Rotation Log tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A48:F48"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add a Recovery Guide tab: where every environment variable lives (#75)
Vercel hides production secrets once saved, so recovery means regenerating,
not restoring. The new tab lists all 36 variables the platform reads, whether
each is a secret or a setting, where it is stored, how to get it back, and
what to know when replacing it, plus a rebuild checklist. It holds no values.
backup-and-recovery.md points to it.

Co-authored-by: AJ Parker <ethnainiceland@gmail.com>
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/alwaysready-api-key-rotation-log.xlsx
+++ b/docs/alwaysready-api-key-rotation-log.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Key Rotation Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Recovery Guide" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -16,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -80,8 +81,25 @@
       <color rgb="001A1A1A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF014D4E"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF014D4E"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +148,23 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF014D4E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -198,11 +231,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB8D4D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB8D4D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB8D4D4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB8D4D4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -257,6 +304,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1214,6 +1281,14 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -1222,4 +1297,1291 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>AlwaysReady Platform: Where every setting lives and how to get it back</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>This sheet holds no secret values, only where each one is stored and how to replace it. Vercel hides production secrets once saved, so the plan if something is lost is to regenerate, never to restore from a copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>Secret or setting</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>Stored in</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>How to get it back</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>What to know when you replace it</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_URL</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>Supabase dashboard, production project (alwaysready-production). Do not use the preview project's address.</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy after changing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SUPABASE_ANON_KEY</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Dashboard → Project Settings → API → Roll</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Logged-in users get a brief auth token refresh. Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>SUPABASE_SERVICE_ROLE_KEY</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Dashboard → Project Settings → API → Roll</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Server-side only. Update Vercel and redeploy straight away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_SECRET_KEY</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>dashboard.stripe.com → Developers → API keys → Roll key</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Stripe supports rolling: create the new key, update Vercel, verify, then revoke the old one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>STRIPE_WEBHOOK_SECRET</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>dashboard.stripe.com → Developers → Webhooks → Roll secret</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>Payment and subscription updates fail to verify until Vercel has the new value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the standard plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only. If a price is recreated its ID changes and Vercel must be updated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>STRIPE_CHARITY_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the charity plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>STRIPE_BETA_PRICE_ID</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Stripe dashboard: the beta plan's price (an ID starting price_).</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>RESEND_API_KEY</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>resend.com → API Keys → Create new → delete old</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>No email sends until Vercel has the new key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>RESEND_FROM_ADDRESS</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Your own sender address. See .env.example for the expected format.</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>RESEND_REPLY_TO</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="inlineStr">
+        <is>
+          <t>Resend</t>
+        </is>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Your own reply-to address. See .env.example.</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>CRON_SECRET</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>No side effects. Vercel sends it to scheduled jobs automatically after a redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>INBOUND_EMAIL_SECRET</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables) AND the Cloudflare Worker that forwards inbound email</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Set the SAME new value in both places, or customer email replies stop reaching the platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>UNSUBSCRIBE_SECRET</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Self-generated</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Not stored anywhere else. Generate a new one: openssl rand -hex 32</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>Every unsubscribe link already sent in past emails stops working, because links are signed with this secret. Only replace if it is lost or leaked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>CLOUDMERSIVE_API_KEY</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>Cloudmersive</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>cloudmersive.com → Account → API Keys → Regenerate</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>Update Vercel and redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_TURNSTILE_SITE_KEY</t>
+        </is>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile: the widget used by the platform. It is a pair with TURNSTILE_SECRET_KEY.</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy. Must belong to the same widget as the secret key.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>TURNSTILE_SECRET_KEY</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare Turnstile</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → Turnstile → select site → rotate secret key</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>Bot check on sign-up forms fails until Vercel matches the widget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SENTRY_DSN</t>
+        </is>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Sentry: the platform project's client key (DSN).</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>Public by design. Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>SENTRY_ORG_SLUG</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Sentry organisation name (alwaysready-platform, per .env.example).</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>SENTRY_AUTH_TOKEN</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Sentry</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>sentry.io → Settings → Auth Tokens → revoke old → create new</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_REST_URL</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Upstash: the Redis database's REST address.</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_REST_TOKEN</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>console.upstash.com → Redis → REST API → Reset token</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>Resetting invalidates existing connections immediately. Update Vercel and redeploy straight away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_MANAGEMENT_API_KEY</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>console.upstash.com → Personal Settings → Developer API → delete old key → create new</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>UPSTASH_MANAGEMENT_EMAIL</t>
+        </is>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Your Upstash account email.</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>UPSTASH_REDIS_DATABASE_ID</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>Upstash</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Upstash: the Redis database's ID.</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>INFRA_VERCEL_TOKEN</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>vercel.com/account/tokens → delete old → create new</t>
+        </is>
+      </c>
+      <c r="F30" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>INFRA_VERCEL_TEAM_ID</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Vercel: your team's ID.</t>
+        </is>
+      </c>
+      <c r="F31" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_API_TOKEN</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → My Profile → API Tokens → delete old → Create Token (Read analytics and logs template)</t>
+        </is>
+      </c>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>Used for the usage card on the Infrastructure page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_ACCOUNT_ID</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare: your account ID.</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>A wrong value here previously blanked the Infrastructure card. Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>CLOUDFLARE_WORKER_NAME</t>
+        </is>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare: the name of the email Worker.</t>
+        </is>
+      </c>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>A wrong value here previously blanked the Infrastructure card. Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>R2_ACCOUNT_ID</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare: your account ID (same as CLOUDFLARE_ACCOUNT_ID).</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>R2_ACCESS_KEY_ID</t>
+        </is>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>dash.cloudflare.com → R2 Object Storage → Manage API Tokens → delete old → Create Account API token (Object Read &amp; Write, scoped to alwaysready-storage-backup)</t>
+        </is>
+      </c>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <t>Nightly Storage backup stops until Vercel has the new pair. /api/health reports it after about 27 hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>R2_SECRET_ACCESS_KEY</t>
+        </is>
+      </c>
+      <c r="B37" s="24" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>Same API token as R2_ACCESS_KEY_ID, regenerate and update both together</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>Comes as a pair with R2_ACCESS_KEY_ID: replace both together.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>R2_BUCKET_NAME</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Cloudflare R2</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>alwaysready-storage-backup (the bucket's name).</t>
+        </is>
+      </c>
+      <c r="F38" s="26" t="inlineStr">
+        <is>
+          <t>Lookup only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>NEXT_PUBLIC_SITE_URL</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Own domain</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>The platform's public address (see .env.example).</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>Baked into the build, so redeploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>SUPERADMIN_EMAIL</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>Setting</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>Own domain</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>Vercel (project environment variables)</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>Your superadmin email (see .env.example).</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to regenerate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>If the Vercel project or its variables are ever lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>0. First, make sure you can log in to every service listed above (keep each two-step recovery code safe). Without access, nothing can be regenerated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>1. Restore or recreate the Vercel project and connect the GitHub repository.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>2. Add every row marked Setting, looking each up as described in "How to get it back".</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>3. For every row marked Secret: regenerate it at its own service, or generate a new value for the self-generated ones, then add it to Vercel. INBOUND_EMAIL_SECRET also goes into the Cloudflare Worker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>4. Redeploy so the new values take effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>5. Check: /api/health returns 200; you can sign in; a test payment event reaches the platform; an email sends; the nightly Storage backup runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>6. Record the new dates in the "Last rotated" column on the Key Rotation Log tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A48:F48"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>